<commit_message>
update summary stats table
</commit_message>
<xml_diff>
--- a/plots/KBS native species phenology summary statisics and environmental optima.xlsx
+++ b/plots/KBS native species phenology summary statisics and environmental optima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbahlai\Dropbox\Active Projects\KBS_LB_phenology\plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBCAC6F7-B6E8-476D-803C-FC814EC762B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E932E970-1932-4532-B517-AF6E1F9D0BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Model statistics" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t>Species</t>
   </si>
@@ -130,6 +130,30 @@
   </si>
   <si>
     <t>Increasing towards zero</t>
+  </si>
+  <si>
+    <t>0.9 (NS)</t>
+  </si>
+  <si>
+    <t>Peak at 642</t>
+  </si>
+  <si>
+    <t>No peak *</t>
+  </si>
+  <si>
+    <t>Peak at 31.8</t>
+  </si>
+  <si>
+    <t>No peak in range of data, slight increase in high and low values</t>
+  </si>
+  <si>
+    <t>Highest in ES</t>
+  </si>
+  <si>
+    <t>Brachiacantha ursina</t>
+  </si>
+  <si>
+    <t>Coleomegilla maculata</t>
   </si>
 </sst>
 </file>
@@ -241,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -268,6 +292,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -747,14 +775,50 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="C4" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E4" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="F4">
+        <v>3.2</v>
+      </c>
+      <c r="G4">
+        <v>2.5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="I4" s="2">
+        <v>3.4</v>
+      </c>
+      <c r="J4" s="17">
+        <v>2.5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="2">
+        <v>3.2</v>
+      </c>
+      <c r="M4" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="N4">
+        <v>8</v>
+      </c>
+      <c r="O4">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+      <c r="A5" s="14" t="s">
+        <v>38</v>
+      </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
@@ -858,7 +922,7 @@
     <col min="4" max="4" width="22.6328125" style="14" customWidth="1"/>
     <col min="5" max="5" width="19.6328125" style="14" customWidth="1"/>
     <col min="6" max="6" width="19.36328125" style="14" customWidth="1"/>
-    <col min="7" max="7" width="23" style="15" customWidth="1"/>
+    <col min="7" max="7" width="23" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -907,22 +971,39 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="B3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="E3" s="15"/>
+      <c r="C3" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="14" t="s">
+        <v>38</v>
+      </c>
       <c r="B4" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="15"/>
       <c r="E4" s="15"/>
+      <c r="G4" s="15"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" s="14" t="s">
@@ -930,6 +1011,7 @@
       </c>
       <c r="C5" s="15"/>
       <c r="E5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B6" s="14" t="s">
@@ -937,6 +1019,7 @@
       </c>
       <c r="C6" s="15"/>
       <c r="E6" s="15"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B7" s="14" t="s">
@@ -944,6 +1027,7 @@
       </c>
       <c r="C7" s="15"/>
       <c r="E7" s="15"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
@@ -951,6 +1035,7 @@
       </c>
       <c r="C8" s="15"/>
       <c r="E8" s="15"/>
+      <c r="G8" s="15"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B9" s="14" t="s">
@@ -958,6 +1043,7 @@
       </c>
       <c r="C9" s="15"/>
       <c r="E9" s="15"/>
+      <c r="G9" s="15"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10" s="14" t="s">
@@ -965,6 +1051,7 @@
       </c>
       <c r="C10" s="15"/>
       <c r="E10" s="15"/>
+      <c r="G10" s="15"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B11" s="14" t="s">
@@ -972,6 +1059,7 @@
       </c>
       <c r="C11" s="15"/>
       <c r="E11" s="15"/>
+      <c r="G11" s="15"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C16" s="14" t="s">

</xml_diff>

<commit_message>
add cmac analysis and compile results
</commit_message>
<xml_diff>
--- a/plots/KBS native species phenology summary statisics and environmental optima.xlsx
+++ b/plots/KBS native species phenology summary statisics and environmental optima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbahlai\Dropbox\Active Projects\KBS_LB_phenology\plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E932E970-1932-4532-B517-AF6E1F9D0BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524C4492-0896-4972-9D86-FB284E4D8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Model statistics" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
   <si>
     <t>Species</t>
   </si>
@@ -154,6 +154,24 @@
   </si>
   <si>
     <t>Coleomegilla maculata</t>
+  </si>
+  <si>
+    <t>Higher activity approaching 0 dd, then lull, then another activity peak near 1128</t>
+  </si>
+  <si>
+    <t>Multiple peaks most pronounced at -1.1, 17.1</t>
+  </si>
+  <si>
+    <t>Highest in maize, followed by wheat</t>
+  </si>
+  <si>
+    <t>peaks at 28.1, 36.5</t>
+  </si>
+  <si>
+    <t>High near zero but slight peak at 46.1 mm</t>
+  </si>
+  <si>
+    <t>Abundance per 5 traps at peak</t>
   </si>
 </sst>
 </file>
@@ -265,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -296,6 +314,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,12 +843,45 @@
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
+      <c r="C5" s="1">
+        <v>0.52</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5.9</v>
+      </c>
+      <c r="E5" s="2">
+        <v>190.8</v>
+      </c>
+      <c r="F5">
+        <v>5.7</v>
+      </c>
+      <c r="G5">
+        <v>22.3</v>
+      </c>
+      <c r="H5" s="2">
+        <v>6.2</v>
+      </c>
+      <c r="I5" s="2">
+        <v>35.79</v>
+      </c>
+      <c r="J5" s="17">
+        <v>6.4</v>
+      </c>
+      <c r="K5">
+        <v>12.2</v>
+      </c>
+      <c r="L5" s="2">
+        <v>6.6</v>
+      </c>
+      <c r="M5" s="2">
+        <v>135.9</v>
+      </c>
+      <c r="N5">
+        <v>8</v>
+      </c>
+      <c r="O5">
+        <v>373</v>
+      </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
@@ -913,7 +967,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8BD8F7D-CC28-428B-AD53-0F2ED668FA0E}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.81640625" style="14" customWidth="1"/>
@@ -923,9 +977,10 @@
     <col min="5" max="5" width="19.6328125" style="14" customWidth="1"/>
     <col min="6" max="6" width="19.36328125" style="14" customWidth="1"/>
     <col min="7" max="7" width="23" style="16" customWidth="1"/>
+    <col min="8" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -947,8 +1002,11 @@
       <c r="G1" s="13" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="H1" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
@@ -970,8 +1028,11 @@
       <c r="G2" s="15" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="H2">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="14" t="s">
         <v>37</v>
       </c>
@@ -993,19 +1054,37 @@
       <c r="G3" s="15" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H3">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="14" t="s">
         <v>38</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="G4" s="15"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="C4" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B5" s="14" t="s">
         <v>7</v>
       </c>
@@ -1013,7 +1092,7 @@
       <c r="E5" s="15"/>
       <c r="G5" s="15"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B6" s="14" t="s">
         <v>8</v>
       </c>
@@ -1021,7 +1100,7 @@
       <c r="E6" s="15"/>
       <c r="G6" s="15"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B7" s="14" t="s">
         <v>9</v>
       </c>
@@ -1029,7 +1108,7 @@
       <c r="E7" s="15"/>
       <c r="G7" s="15"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
         <v>10</v>
       </c>
@@ -1037,7 +1116,7 @@
       <c r="E8" s="15"/>
       <c r="G8" s="15"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B9" s="14" t="s">
         <v>11</v>
       </c>
@@ -1045,7 +1124,7 @@
       <c r="E9" s="15"/>
       <c r="G9" s="15"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B10" s="14" t="s">
         <v>12</v>
       </c>
@@ -1053,7 +1132,7 @@
       <c r="E10" s="15"/>
       <c r="G10" s="15"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B11" s="14" t="s">
         <v>13</v>
       </c>
@@ -1061,7 +1140,7 @@
       <c r="E11" s="15"/>
       <c r="G11" s="15"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C16" s="14" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
add cstig analysis, checked up to line 1756
</commit_message>
<xml_diff>
--- a/plots/KBS native species phenology summary statisics and environmental optima.xlsx
+++ b/plots/KBS native species phenology summary statisics and environmental optima.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbahlai\Dropbox\Active Projects\KBS_LB_phenology\plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524C4492-0896-4972-9D86-FB284E4D8D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4508DEDB-99F2-4564-BBF5-60CBF8513119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
+    <workbookView xWindow="37440" yWindow="1620" windowWidth="18480" windowHeight="8580" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Model statistics" sheetId="1" r:id="rId1"/>
@@ -156,9 +156,6 @@
     <t>Coleomegilla maculata</t>
   </si>
   <si>
-    <t>Higher activity approaching 0 dd, then lull, then another activity peak near 1128</t>
-  </si>
-  <si>
     <t>Multiple peaks most pronounced at -1.1, 17.1</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>Abundance per 5 traps at peak</t>
+  </si>
+  <si>
+    <t>Higher activity approaching 0 dd, then low, then another activity peak near 1128</t>
   </si>
 </sst>
 </file>
@@ -1003,7 +1003,7 @@
         <v>19</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -1066,19 +1066,19 @@
         <v>6</v>
       </c>
       <c r="C4" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="14" t="s">
+      <c r="G4" s="15" t="s">
         <v>40</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>41</v>
       </c>
       <c r="H4">
         <v>3.2</v>

</xml_diff>

<commit_message>
Updated with additional LB
</commit_message>
<xml_diff>
--- a/plots/KBS native species phenology summary statisics and environmental optima.xlsx
+++ b/plots/KBS native species phenology summary statisics and environmental optima.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbahlai\Dropbox\Active Projects\KBS_LB_phenology\plots\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aee9d26e930415cd/Documents/GitHub/KBS_LB_phenology/plots/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4508DEDB-99F2-4564-BBF5-60CBF8513119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="195" documentId="13_ncr:1_{4508DEDB-99F2-4564-BBF5-60CBF8513119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD74CE61-49B5-462E-9E89-8F8B33283170}"/>
   <bookViews>
-    <workbookView xWindow="37440" yWindow="1620" windowWidth="18480" windowHeight="8580" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{11554A19-541E-4013-A930-2B63B96F32FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Model statistics" sheetId="1" r:id="rId1"/>
     <sheet name="Optimal values" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="92">
   <si>
     <t>Species</t>
   </si>
@@ -172,6 +173,147 @@
   </si>
   <si>
     <t>Higher activity approaching 0 dd, then low, then another activity peak near 1128</t>
+  </si>
+  <si>
+    <t>2.2(NS)</t>
+  </si>
+  <si>
+    <t>1.2(NS)</t>
+  </si>
+  <si>
+    <t>0.4(NS)</t>
+  </si>
+  <si>
+    <t>Highest in deciduous followed by poplar</t>
+  </si>
+  <si>
+    <t>Multiple peaks most pronounced at -0.8, 13.8*</t>
+  </si>
+  <si>
+    <t>peaks at 26 and 33.4*</t>
+  </si>
+  <si>
+    <t>peak at 43.6 mm*</t>
+  </si>
+  <si>
+    <t>Higher activity approaching 0 dd, then low, then another activity peak near 938</t>
+  </si>
+  <si>
+    <t>0.9(NS)</t>
+  </si>
+  <si>
+    <t>0.2(NS)</t>
+  </si>
+  <si>
+    <t>1.5(NS)</t>
+  </si>
+  <si>
+    <t>1(NS)</t>
+  </si>
+  <si>
+    <t>Highest in poplar</t>
+  </si>
+  <si>
+    <t>Lower activity approaching 0 dd, then an increase until a peak near 1148</t>
+  </si>
+  <si>
+    <t>peak at 117.9 mm</t>
+  </si>
+  <si>
+    <t>peaks at 21.5 and 34.4*</t>
+  </si>
+  <si>
+    <t>peak at 14.2</t>
+  </si>
+  <si>
+    <t>2.6(NS)</t>
+  </si>
+  <si>
+    <t>2.3(NS)</t>
+  </si>
+  <si>
+    <t>Highest in alfalfa, coniferous, deciduous, and successional</t>
+  </si>
+  <si>
+    <t>Higher activity approaching 0 then peak at 582 dd, then increase until 1400*</t>
+  </si>
+  <si>
+    <t>No peak in range of data, slope levels off as precip increases*</t>
+  </si>
+  <si>
+    <t>peaks at 25.1 and 32.6*</t>
+  </si>
+  <si>
+    <t>peak at 13.1*</t>
+  </si>
+  <si>
+    <t>Highest in deciduous followed by wheat</t>
+  </si>
+  <si>
+    <t>Lower activity approaching 0 dd, then an increase until a peak near 1069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High near 0 but slight peak at 45.2 mm </t>
+  </si>
+  <si>
+    <t>peak at 33.2</t>
+  </si>
+  <si>
+    <t>peak at 15.8</t>
+  </si>
+  <si>
+    <t>Wheat</t>
+  </si>
+  <si>
+    <t>Peak at 62.7 mm</t>
+  </si>
+  <si>
+    <t>1.6(NS)</t>
+  </si>
+  <si>
+    <t>1.8(NS)</t>
+  </si>
+  <si>
+    <t>2.5(NS)</t>
+  </si>
+  <si>
+    <t>peak at 14*</t>
+  </si>
+  <si>
+    <t>Peaks at 662 and 838*</t>
+  </si>
+  <si>
+    <t>2(NS)</t>
+  </si>
+  <si>
+    <t>peak at 13.8*</t>
+  </si>
+  <si>
+    <t>peaks at 57.7 and 104.8*</t>
+  </si>
+  <si>
+    <t>Highest in  wheat and then ES</t>
+  </si>
+  <si>
+    <t>peak at 26.1 (minimum peak)</t>
+  </si>
+  <si>
+    <t>Peak at 426 dd, then constant increase in slope</t>
+  </si>
+  <si>
+    <t>no peaks</t>
+  </si>
+  <si>
+    <t>peak at 30.6 mm*</t>
+  </si>
+  <si>
+    <t>no peaks*</t>
+  </si>
+  <si>
+    <t>peak at 26.7</t>
+  </si>
+  <si>
+    <t>peaks at 722 and 1133*</t>
   </si>
 </sst>
 </file>
@@ -283,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -310,11 +452,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -332,6 +470,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -817,7 +959,7 @@
       <c r="I4" s="2">
         <v>3.4</v>
       </c>
-      <c r="J4" s="17">
+      <c r="J4">
         <v>2.5</v>
       </c>
       <c r="K4" t="s">
@@ -864,7 +1006,7 @@
       <c r="I5" s="2">
         <v>35.79</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5">
         <v>6.4</v>
       </c>
       <c r="K5">
@@ -887,78 +1029,309 @@
       <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
+      <c r="C6" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2.7</v>
+      </c>
+      <c r="E6" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="F6">
+        <v>3.1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="2">
+        <v>3</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J6">
+        <v>3.2</v>
+      </c>
+      <c r="K6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L6" s="2">
+        <v>3.3</v>
+      </c>
+      <c r="M6" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="N6">
+        <v>8</v>
+      </c>
+      <c r="O6">
+        <v>11.6</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="C7" s="1">
+        <v>0.13</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7">
+        <v>1.7</v>
+      </c>
+      <c r="G7" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="J7">
+        <v>1.7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>55</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="M7" s="2">
+        <v>4.8</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="C8" s="1">
+        <v>0.26</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4.3</v>
+      </c>
+      <c r="E8" s="2">
+        <v>63.5</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8">
+        <v>5.2</v>
+      </c>
+      <c r="H8" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8">
+        <v>4.5</v>
+      </c>
+      <c r="K8">
+        <v>3</v>
+      </c>
+      <c r="L8" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="M8" s="2">
+        <v>48.1</v>
+      </c>
+      <c r="N8">
+        <v>8</v>
+      </c>
+      <c r="O8">
+        <v>135.5</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="C9" s="1">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9">
+        <v>1.9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J9">
+        <v>1.6</v>
+      </c>
+      <c r="K9" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" s="2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="M9" s="2">
+        <v>48.5</v>
+      </c>
+      <c r="N9">
+        <v>4</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="C10" s="1">
+        <v>0.18</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2.4</v>
+      </c>
+      <c r="E10" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="F10">
+        <v>2.5</v>
+      </c>
+      <c r="G10">
+        <v>2.9</v>
+      </c>
+      <c r="H10" s="2">
+        <v>2.9</v>
+      </c>
+      <c r="I10" s="2">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="J10">
+        <v>2.1</v>
+      </c>
+      <c r="K10">
+        <v>11.5</v>
+      </c>
+      <c r="L10" s="2">
+        <v>3</v>
+      </c>
+      <c r="M10" s="2">
+        <v>10.3</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+      <c r="C11" s="1">
+        <v>0.23</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11">
+        <v>2.6</v>
+      </c>
+      <c r="G11">
+        <v>2.6</v>
+      </c>
+      <c r="H11" s="2">
+        <v>2.8</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J11">
+        <v>2.4</v>
+      </c>
+      <c r="K11" t="s">
+        <v>76</v>
+      </c>
+      <c r="L11" s="2">
+        <v>2.7</v>
+      </c>
+      <c r="M11" s="2">
+        <v>50.7</v>
+      </c>
+      <c r="N11">
+        <v>8</v>
+      </c>
+      <c r="O11">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="C12" s="1">
+        <v>0.16</v>
+      </c>
+      <c r="D12" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="E12" s="2">
+        <v>12.1</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="I12" s="2">
+        <v>7.9</v>
+      </c>
+      <c r="J12">
+        <v>4</v>
+      </c>
+      <c r="K12" t="s">
+        <v>55</v>
+      </c>
+      <c r="L12" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="M12" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="N12">
+        <v>8</v>
+      </c>
+      <c r="O12">
+        <v>56.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -976,11 +1349,11 @@
     <col min="4" max="4" width="22.6328125" style="14" customWidth="1"/>
     <col min="5" max="5" width="19.6328125" style="14" customWidth="1"/>
     <col min="6" max="6" width="19.36328125" style="14" customWidth="1"/>
-    <col min="7" max="7" width="23" style="16" customWidth="1"/>
+    <col min="7" max="7" width="23" style="14" customWidth="1"/>
     <col min="8" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1375,7 @@
       <c r="G1" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="16" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1084,61 +1457,166 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B5" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="G5" s="15"/>
+      <c r="C5" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B6" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="G6" s="15"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C6" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="G7" s="15"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C7" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="G8" s="15"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C8" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B9" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="C9" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="G10" s="15"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C10" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="B11" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="C11" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="H11">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C16" s="14" t="s">

</xml_diff>